<commit_message>
servicio cargar descuento excel creado, permite guardar registros, pendiente guardar
</commit_message>
<xml_diff>
--- a/public/format/plantilla-descuentos.xlsx
+++ b/public/format/plantilla-descuentos.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROGRAMACION\NODEJS\rest-sgd\public\format\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED1AD4C-592D-423D-8495-B04D8573C7ED}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB607624-8926-4CB4-BE72-2FB5AD99D6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{49D0E559-6948-42F6-8991-0DDDC8C8E4D1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{49D0E559-6948-42F6-8991-0DDDC8C8E4D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="otra-hoja" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -229,7 +228,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -258,14 +257,6 @@
       <name val="Tahoma"/>
       <charset val="1"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -287,10 +278,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -606,22 +596,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87B629FE-7C12-4EAD-8114-BB5BC3114295}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -656,7 +646,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B2">
         <v>1</v>
       </c>
@@ -690,18 +680,4 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE89477-6F3A-4F38-B853-C580E58B56D1}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fomulario cargue descuentos finalizado, se valida eliminacion de codigos
</commit_message>
<xml_diff>
--- a/public/format/plantilla-descuentos.xlsx
+++ b/public/format/plantilla-descuentos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROGRAMACION\NODEJS\rest-sgd\public\format\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB607624-8926-4CB4-BE72-2FB5AD99D6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9530F98A-4FF2-426B-B5AF-7CECC7F5565B}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{49D0E559-6948-42F6-8991-0DDDC8C8E4D1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{49D0E559-6948-42F6-8991-0DDDC8C8E4D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -30,6 +30,30 @@
     <author>Dvn</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{91131E17-954C-402A-9159-190DCD352AC6}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Dvn:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+dejar vacio</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="B1" authorId="0" shapeId="0" xr:uid="{531A9B30-AB78-438E-AB71-153C7011BCDA}">
       <text>
         <r>
@@ -78,6 +102,30 @@
 2: APROBADO
 3: RECHAZADO
 4: FACTURADO</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{A6E24D06-79F8-4C42-963C-0BA93AA40B33}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Dvn:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+si no hay codigo, dejar vacio</t>
         </r>
       </text>
     </comment>
@@ -106,7 +154,10 @@
 3: BENEFICIO GENERACION E
 4: MATRICULA DE HONOR
 5: ALVARO ULCUE CHOCUE
-</t>
+6: COOTEP SUPERIOR
+7: POBLACION VICTIMA MEN
+8: OTRO
+9: GOB NACIONAL Y DPTAL ESTRATO 1,2,3</t>
         </r>
       </text>
     </comment>
@@ -595,23 +646,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87B629FE-7C12-4EAD-8114-BB5BC3114295}">
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -644,35 +695,6 @@
       </c>
       <c r="K1" s="1" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>18131047</v>
-      </c>
-      <c r="E2">
-        <v>597311</v>
-      </c>
-      <c r="F2">
-        <v>3</v>
-      </c>
-      <c r="G2">
-        <v>0.4</v>
-      </c>
-      <c r="H2">
-        <v>39</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>